<commit_message>
fix import of users
</commit_message>
<xml_diff>
--- a/public/example.xlsx
+++ b/public/example.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\admin\Documents\workspace\Laravel\cyfgs-brocon-financial-assistance\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBE724AA-A138-4B82-829A-F082CA0C6DBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EA85666-7767-44C2-A3FE-263400CF0693}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="40">
   <si>
     <t>Name</t>
   </si>
@@ -104,6 +104,42 @@
   </si>
   <si>
     <t>bright@gmail.com</t>
+  </si>
+  <si>
+    <t>Username</t>
+  </si>
+  <si>
+    <t>peterjerry</t>
+  </si>
+  <si>
+    <t>lewisshalla</t>
+  </si>
+  <si>
+    <t>patterson</t>
+  </si>
+  <si>
+    <t>abramjoe</t>
+  </si>
+  <si>
+    <t>billclinton</t>
+  </si>
+  <si>
+    <t>Nforbi Nji</t>
+  </si>
+  <si>
+    <t>nforbinji</t>
+  </si>
+  <si>
+    <t>brightpat</t>
+  </si>
+  <si>
+    <t>Williams Kennedy</t>
+  </si>
+  <si>
+    <t>williamkennedy@gmail.com</t>
+  </si>
+  <si>
+    <t>williamskennedy</t>
   </si>
 </sst>
 </file>
@@ -391,7 +427,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultColWidth="12.7109375" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.5703125" customWidth="1"/>
@@ -399,7 +435,7 @@
     <col min="3" max="3" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -418,8 +454,11 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="G1" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>6</v>
       </c>
@@ -438,8 +477,11 @@
       <c r="F2" s="3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="G2" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>14</v>
       </c>
@@ -458,8 +500,11 @@
       <c r="F3" s="3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G3" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -478,8 +523,11 @@
       <c r="F4" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -498,8 +546,11 @@
       <c r="F5" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>24</v>
       </c>
@@ -518,10 +569,13 @@
       <c r="F6" s="3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G6" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>22</v>
@@ -538,8 +592,11 @@
       <c r="F7" s="3" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G7" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>26</v>
       </c>
@@ -558,16 +615,19 @@
       <c r="F8" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G8" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="C9" s="2">
-        <v>678934023</v>
+        <v>670034023</v>
       </c>
       <c r="D9" t="s">
         <v>8</v>
@@ -577,6 +637,9 @@
       </c>
       <c r="F9" t="s">
         <v>23</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>